<commit_message>
fixed the issue of salary slip for employee, mailing, validations
</commit_message>
<xml_diff>
--- a/client/public/samples/bulk-attendance-sample.xlsx
+++ b/client/public/samples/bulk-attendance-sample.xlsx
@@ -4,89 +4,101 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="JULY" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
-  <si>
-    <t>employeeId</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>date</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>checkIn</t>
-  </si>
-  <si>
-    <t>checkOut</t>
-  </si>
-  <si>
-    <t>EMP45872</t>
-  </si>
-  <si>
-    <t>rahul.kumar@xyz.com</t>
-  </si>
-  <si>
-    <t>2026-07-05</t>
-  </si>
-  <si>
-    <t>Present</t>
-  </si>
-  <si>
-    <t>09:30</t>
-  </si>
-  <si>
-    <t>18:30</t>
-  </si>
-  <si>
-    <t>EMP45873</t>
-  </si>
-  <si>
-    <t>amit.patel@xyz.com</t>
-  </si>
-  <si>
-    <t>Absent</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="25">
+  <si>
+    <t>MIRUS MEDSCIENCES PRIVATE LIMITED - STAFF ATTENDANCE FOR THE MONTH OF JULY 2026</t>
+  </si>
+  <si>
+    <t>S.No.</t>
+  </si>
+  <si>
+    <t>Emp.Id</t>
+  </si>
+  <si>
+    <t>Name of The Employee</t>
+  </si>
+  <si>
+    <t>Contact No.</t>
+  </si>
+  <si>
+    <t>WED</t>
+  </si>
+  <si>
+    <t>THUR</t>
+  </si>
+  <si>
+    <t>FRI</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>SUN</t>
+  </si>
+  <si>
+    <t>MON</t>
+  </si>
+  <si>
+    <t>TUE</t>
+  </si>
+  <si>
+    <t>PD</t>
+  </si>
+  <si>
+    <t>AD</t>
+  </si>
+  <si>
+    <t>TD</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>EMP45874</t>
-  </si>
-  <si>
-    <t>neha.gupta@xyz.com</t>
-  </si>
-  <si>
-    <t>Half-Day</t>
-  </si>
-  <si>
-    <t>13:30</t>
+    <t>MMS0011</t>
+  </si>
+  <si>
+    <t>Sample Employee One</t>
+  </si>
+  <si>
+    <t>98765 43210</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>MMS0012</t>
+  </si>
+  <si>
+    <t>Sample Employee Two</t>
+  </si>
+  <si>
+    <t>91234 56789</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -109,9 +121,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,90 +462,476 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="6" width="18" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="D2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E2" t="s">
         <v>5</v>
       </c>
+      <c r="F2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" t="s">
+        <v>7</v>
+      </c>
+      <c r="O2" t="s">
+        <v>8</v>
+      </c>
+      <c r="P2" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>10</v>
+      </c>
+      <c r="R2" t="s">
+        <v>11</v>
+      </c>
+      <c r="S2" t="s">
+        <v>5</v>
+      </c>
+      <c r="T2" t="s">
+        <v>6</v>
+      </c>
+      <c r="U2" t="s">
+        <v>7</v>
+      </c>
+      <c r="V2" t="s">
+        <v>8</v>
+      </c>
+      <c r="W2" t="s">
+        <v>9</v>
+      </c>
+      <c r="X2" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>6</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>7</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>7</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>12</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>13</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="K3">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="L3">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="M3">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="N3">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="O3">
         <v>11</v>
       </c>
+      <c r="P3">
+        <v>12</v>
+      </c>
+      <c r="Q3">
+        <v>13</v>
+      </c>
+      <c r="R3">
+        <v>14</v>
+      </c>
+      <c r="S3">
+        <v>15</v>
+      </c>
+      <c r="T3">
+        <v>16</v>
+      </c>
+      <c r="U3">
+        <v>17</v>
+      </c>
+      <c r="V3">
+        <v>18</v>
+      </c>
+      <c r="W3">
+        <v>19</v>
+      </c>
+      <c r="X3">
+        <v>20</v>
+      </c>
+      <c r="Y3">
+        <v>21</v>
+      </c>
+      <c r="Z3">
+        <v>22</v>
+      </c>
+      <c r="AA3">
+        <v>23</v>
+      </c>
+      <c r="AB3">
+        <v>24</v>
+      </c>
+      <c r="AC3">
+        <v>25</v>
+      </c>
+      <c r="AD3">
+        <v>26</v>
+      </c>
+      <c r="AE3">
+        <v>27</v>
+      </c>
+      <c r="AF3">
+        <v>28</v>
+      </c>
+      <c r="AG3">
+        <v>29</v>
+      </c>
+      <c r="AH3">
+        <v>30</v>
+      </c>
+      <c r="AI3">
+        <v>31</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>15</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>15</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
       </c>
       <c r="D4" t="s">
         <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
         <v>19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" t="s">
+        <v>19</v>
+      </c>
+      <c r="L4" t="s">
+        <v>19</v>
+      </c>
+      <c r="M4" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" t="s">
+        <v>19</v>
+      </c>
+      <c r="O4" t="s">
+        <v>19</v>
+      </c>
+      <c r="P4" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>19</v>
+      </c>
+      <c r="R4" t="s">
+        <v>19</v>
+      </c>
+      <c r="S4" t="s">
+        <v>19</v>
+      </c>
+      <c r="T4" t="s">
+        <v>19</v>
+      </c>
+      <c r="U4" t="s">
+        <v>19</v>
+      </c>
+      <c r="V4" t="s">
+        <v>20</v>
+      </c>
+      <c r="W4" t="s">
+        <v>21</v>
+      </c>
+      <c r="X4" t="s">
+        <v>19</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>19</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AJ4">
+        <v>0</v>
+      </c>
+      <c r="AK4">
+        <v>0</v>
+      </c>
+      <c r="AL4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" t="s">
+        <v>19</v>
+      </c>
+      <c r="K5" t="s">
+        <v>19</v>
+      </c>
+      <c r="L5" t="s">
+        <v>19</v>
+      </c>
+      <c r="M5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N5" t="s">
+        <v>19</v>
+      </c>
+      <c r="O5" t="s">
+        <v>19</v>
+      </c>
+      <c r="P5" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>19</v>
+      </c>
+      <c r="R5" t="s">
+        <v>19</v>
+      </c>
+      <c r="S5" t="s">
+        <v>19</v>
+      </c>
+      <c r="T5" t="s">
+        <v>19</v>
+      </c>
+      <c r="U5" t="s">
+        <v>19</v>
+      </c>
+      <c r="V5" t="s">
+        <v>19</v>
+      </c>
+      <c r="W5" t="s">
+        <v>19</v>
+      </c>
+      <c r="X5" t="s">
+        <v>19</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>19</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AJ5">
+        <v>0</v>
+      </c>
+      <c r="AK5">
+        <v>0</v>
+      </c>
+      <c r="AL5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>